<commit_message>
Abandonar Command solo mvc por ahora
</commit_message>
<xml_diff>
--- a/mi-proyecto/docs/TablasInventario.xlsx
+++ b/mi-proyecto/docs/TablasInventario.xlsx
@@ -5,26 +5,24 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="producto" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="historico de productos" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="hitorico de ventas" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="lote" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="ventas" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="detalle de la venta" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="cliente" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="historico credito" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="alertas" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="alertas" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">alertas!$A$1:$B$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">alertas!$A$1:$B$1</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">cliente!$A$1:$F$3</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'detalle de la venta'!$A$1:$D$10</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'historico credito'!$A$1:$E$6</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'historico de productos'!$A$1:$G$22</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'hitorico de ventas'!$A$1:$F$6</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">lote!$A$1:$G$22</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">producto!$A$1:$H$20</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm._FilterDatabase_1" vbProcedure="false">'historico de productos'!$A$1:$G$20</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">ventas!$A$1:$F$6</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm._FilterDatabase_1" vbProcedure="false">lote!$A$1:$G$20</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="76">
   <si>
     <t xml:space="preserve">Id</t>
   </si>
@@ -95,6 +93,12 @@
     <t xml:space="preserve">gr</t>
   </si>
   <si>
+    <t xml:space="preserve">Arroz x 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arroz Boluga</t>
+  </si>
+  <si>
     <t xml:space="preserve">Diana</t>
   </si>
   <si>
@@ -245,32 +249,33 @@
     <t xml:space="preserve">tp@email.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Id Cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Id Venta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Credito</t>
-  </si>
-  <si>
     <t xml:space="preserve">titulo</t>
   </si>
   <si>
     <t xml:space="preserve">cuerpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la RAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agotado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vencimineto</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="167" formatCode="hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yy\ hh:mm"/>
+    <numFmt numFmtId="168" formatCode="hh:mm:ss"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -310,6 +315,13 @@
       <u val="single"/>
       <sz val="10"/>
       <color rgb="FF0000EE"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC9211E"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -364,7 +376,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -409,15 +421,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -430,7 +458,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -450,6 +478,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0000EE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC9211E"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -509,7 +545,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -539,10 +575,6 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -788,8 +820,7 @@
         <v>17</v>
       </c>
       <c r="E4" s="3" t="n">
-        <f aca="false">30*500</f>
-        <v>15000</v>
+        <v>500</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>18</v>
@@ -801,7 +832,7 @@
         <v>200</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>50</v>
@@ -816,25 +847,25 @@
         <v>78545457</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>5000</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>50</v>
@@ -852,13 +883,13 @@
         <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>13</v>
@@ -882,16 +913,16 @@
         <v>78545459</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>13</v>
@@ -913,16 +944,16 @@
         <v>78545460</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>13</v>
@@ -944,16 +975,16 @@
         <v>78545461</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>1000</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>13</v>
@@ -975,10 +1006,10 @@
         <v>78545462</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>6</v>
@@ -1006,10 +1037,10 @@
         <v>78545463</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>12</v>
@@ -1037,16 +1068,16 @@
         <v>78545464</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>250</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>13</v>
@@ -1066,10 +1097,10 @@
         <v>78545465</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>6</v>
@@ -1095,10 +1126,10 @@
         <v>78545466</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>24</v>
@@ -1124,10 +1155,10 @@
         <v>78545467</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>6</v>
@@ -1153,16 +1184,16 @@
         <v>78545468</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>250</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>13</v>
@@ -1182,16 +1213,16 @@
         <v>78545469</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>250</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>13</v>
@@ -1211,16 +1242,16 @@
         <v>78545470</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>250</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>13</v>
@@ -1240,10 +1271,10 @@
         <v>78545471</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>50</v>
@@ -1269,7 +1300,7 @@
         <v>78545472</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="3" t="n">
@@ -1306,7 +1337,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.2"/>
@@ -1325,25 +1356,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1356,7 +1387,7 @@
       </c>
       <c r="C2" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>1459</v>
+        <v>7853</v>
       </c>
       <c r="D2" s="9" t="n">
         <v>46219</v>
@@ -1381,7 +1412,7 @@
       </c>
       <c r="C3" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>8671</v>
+        <v>7278</v>
       </c>
       <c r="D3" s="9" t="n">
         <v>46220</v>
@@ -1407,7 +1438,7 @@
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>7411</v>
+        <v>1435</v>
       </c>
       <c r="D4" s="9" t="n">
         <v>46221</v>
@@ -1433,7 +1464,7 @@
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>3311</v>
+        <v>9187</v>
       </c>
       <c r="D5" s="9" t="n">
         <v>46222</v>
@@ -1459,7 +1490,7 @@
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>7083</v>
+        <v>7450</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>46223</v>
@@ -1485,7 +1516,7 @@
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>6099</v>
+        <v>4153</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>46224</v>
@@ -1511,7 +1542,7 @@
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>4380</v>
+        <v>1664</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>46225</v>
@@ -1537,7 +1568,7 @@
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>9722</v>
+        <v>1947</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>46226</v>
@@ -1563,7 +1594,7 @@
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>9856</v>
+        <v>3926</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>46227</v>
@@ -1589,7 +1620,7 @@
       </c>
       <c r="C11" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>1499</v>
+        <v>6669</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>46228</v>
@@ -1615,7 +1646,7 @@
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>8761</v>
+        <v>2229</v>
       </c>
       <c r="D12" s="9" t="n">
         <v>46229</v>
@@ -1641,7 +1672,7 @@
       </c>
       <c r="C13" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>2226</v>
+        <v>4977</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>46230</v>
@@ -1667,7 +1698,7 @@
       </c>
       <c r="C14" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>5255</v>
+        <v>2811</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>46231</v>
@@ -1693,7 +1724,7 @@
       </c>
       <c r="C15" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>3851</v>
+        <v>5443</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>46232</v>
@@ -1719,7 +1750,7 @@
       </c>
       <c r="C16" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>4477</v>
+        <v>1698</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>46233</v>
@@ -1743,7 +1774,7 @@
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>2784</v>
+        <v>3611</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>46234</v>
@@ -1767,7 +1798,7 @@
       </c>
       <c r="C18" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>8061</v>
+        <v>2505</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>46235</v>
@@ -1791,7 +1822,7 @@
       </c>
       <c r="C19" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>6228</v>
+        <v>2872</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>46236</v>
@@ -1815,7 +1846,7 @@
       </c>
       <c r="C20" s="8" t="n">
         <f aca="false">RANDBETWEEN(999,9999)</f>
-        <v>5694</v>
+        <v>2520</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>46237</v>
@@ -1840,7 +1871,7 @@
       </c>
       <c r="C21" s="8" t="n">
         <f aca="false">C3</f>
-        <v>8671</v>
+        <v>7278</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>46220</v>
@@ -1866,7 +1897,7 @@
       </c>
       <c r="C22" s="8" t="n">
         <f aca="false">C3</f>
-        <v>8671</v>
+        <v>7278</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>46220</v>
@@ -1880,6 +1911,15 @@
       <c r="G22" s="3" t="n">
         <v>-3000</v>
       </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G22"/>
@@ -1915,19 +1955,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1940,14 +1980,14 @@
       <c r="C2" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="D2" s="11" t="n">
+      <c r="D2" s="13" t="n">
         <v>46023</v>
       </c>
-      <c r="E2" s="12" t="n">
+      <c r="E2" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1962,7 +2002,7 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1978,7 +2018,7 @@
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1988,7 +2028,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1998,7 +2038,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2145,16 +2185,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2362,19 +2402,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2382,13 +2422,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C2" s="5" t="n">
         <v>10000000</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>66</v>
+      <c r="D2" s="15" t="s">
+        <v>68</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>3552277777</v>
@@ -2403,13 +2443,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C3" s="5" t="n">
         <v>12555555</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>68</v>
+      <c r="D3" s="15" t="s">
+        <v>70</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>3225448454</v>
@@ -2577,235 +2617,34 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="9.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="6" style="1" width="9.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1125" min="1025" style="1" width="7.52"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>-70000</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
-        <f aca="false">A2+1</f>
-        <v>2</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <autoFilter ref="A1:E6"/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.700694444444445" right="0.700694444444445" top="1.05208333333333" bottom="1.05208333333333" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="17" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5"/>
+      <c r="A2" s="5" t="s">
+        <v>74</v>
+      </c>
       <c r="B2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
+      <c r="A3" s="5" t="s">
+        <v>75</v>
+      </c>
       <c r="B3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>